<commit_message>
fv charm & gens 3days
</commit_message>
<xml_diff>
--- a/gu_in/ItemTimer.edf/TimerItem.xlsx
+++ b/gu_in/ItemTimer.edf/TimerItem.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4481996-DC07-4248-80A5-1430348954C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80CB4AC-5E2E-4C61-B34C-A740B65C24B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TimerItem" sheetId="1" r:id="rId1"/>
@@ -1776,9 +1776,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1816,9 +1816,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1851,9 +1851,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1886,9 +1903,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4472,7 +4506,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirval01</v>
@@ -4487,7 +4521,7 @@
         <v>604800</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tiaqsa04</v>
@@ -4502,7 +4536,7 @@
         <v>2592000</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tiaqsa05</v>
@@ -4517,7 +4551,7 @@
         <v>2592000</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tiaqsa06</v>
@@ -4532,7 +4566,7 @@
         <v>2592000</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tiaqsa07</v>
@@ -4547,7 +4581,7 @@
         <v>2592000</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tiiqsa04</v>
@@ -4562,7 +4596,7 @@
         <v>2592000</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tiiqsa05</v>
@@ -4577,7 +4611,7 @@
         <v>2592000</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm46</v>
@@ -4589,10 +4623,11 @@
         <v>2</v>
       </c>
       <c r="D168" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F168" s="2"/>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm47</v>
@@ -4604,10 +4639,11 @@
         <v>2</v>
       </c>
       <c r="D169" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F169" s="2"/>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm48</v>
@@ -4619,10 +4655,11 @@
         <v>2</v>
       </c>
       <c r="D170" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F170" s="2"/>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm49</v>
@@ -4634,10 +4671,11 @@
         <v>2</v>
       </c>
       <c r="D171" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F171" s="2"/>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm50</v>
@@ -4649,10 +4687,11 @@
         <v>2</v>
       </c>
       <c r="D172" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F172" s="2"/>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm51</v>
@@ -4664,10 +4703,11 @@
         <v>2</v>
       </c>
       <c r="D173" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F173" s="2"/>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm52</v>
@@ -4679,10 +4719,11 @@
         <v>2</v>
       </c>
       <c r="D174" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F174" s="2"/>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm53</v>
@@ -4694,10 +4735,11 @@
         <v>2</v>
       </c>
       <c r="D175" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F175" s="2"/>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm54</v>
@@ -4709,10 +4751,11 @@
         <v>2</v>
       </c>
       <c r="D176" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F176" s="2"/>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm55</v>
@@ -4724,10 +4767,11 @@
         <v>2</v>
       </c>
       <c r="D177" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F177" s="2"/>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm56</v>
@@ -4739,10 +4783,11 @@
         <v>2</v>
       </c>
       <c r="D178" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F178" s="2"/>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tirchm57</v>
@@ -4754,10 +4799,11 @@
         <v>2</v>
       </c>
       <c r="D179" s="1">
-        <v>432000</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259200</v>
+      </c>
+      <c r="F179" s="2"/>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy01</v>
@@ -4772,7 +4818,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy02</v>
@@ -4787,7 +4833,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy03</v>
@@ -4802,7 +4848,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy04</v>
@@ -4817,7 +4863,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy05</v>
@@ -4832,7 +4878,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy06</v>
@@ -4847,7 +4893,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy07</v>
@@ -4862,7 +4908,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy08</v>
@@ -4877,7 +4923,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy09</v>
@@ -4892,7 +4938,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy10</v>
@@ -4907,7 +4953,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy11</v>
@@ -4922,7 +4968,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy12</v>
@@ -4937,7 +4983,7 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="str">
         <f t="shared" si="2"/>
         <v>tihemy13</v>

</xml_diff>